<commit_message>
fix: replace Excel 365 functions (XLOOKUP/IFS) with LibreOffice-compatible INDEX/MATCH and nested IF
This fixes the #NAME? error in B14 (rating Finanziaria) and related grade/fido
calculations that were failing in LibreOffice < 24.8 because XLOOKUP and IFS are
not natively supported. The template now works correctly in both Excel and LibreOffice.

Changes:
- Replace _xlfn.XLOOKUP with INDEX/MATCH in Input!H90, I90, J90, I92, D83 and Report!B14
- Replace _xlfn.IFS with nested IF in Input!H89, I89, J89
- Move B14 (Finanziaria rating) from formula to Python-calculated value (build_report.py, metrics.py, narrative.py)
- This ensures consistent rating calculation across all three dimensions (Reddituale, Finanziaria, Patrimoniale)

The fix is backward-compatible with Excel while enabling support for LibreOffice and claude.ai/web environments.

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plugins/fs-analysis/skills/analyzing-financial-statements/assets/template.xlsx
+++ b/plugins/fs-analysis/skills/analyzing-financial-statements/assets/template.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="Questa_cartella_di_lavoro"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Input" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Input" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Report" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Report'!$A$1:$D$185</definedName>
@@ -1378,7 +1378,7 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <plotArea>
       <layout/>
@@ -1388,7 +1388,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1396,10 +1396,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="00B050"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:ln w="19050">
                 <a:solidFill>
                   <a:schemeClr val="lt1"/>
                 </a:solidFill>
@@ -1411,13 +1411,13 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:schemeClr val="tx2">
                   <a:lumMod val="40000"/>
                   <a:lumOff val="60000"/>
                 </a:schemeClr>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:ln w="19050">
                 <a:solidFill>
                   <a:schemeClr val="lt1"/>
                 </a:solidFill>
@@ -1429,8 +1429,8 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:noFill/>
+              <a:ln w="19050">
                 <a:solidFill>
                   <a:schemeClr val="lt1"/>
                 </a:solidFill>
@@ -1474,8 +1474,8 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:noFill/>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:noFill/>
       <a:prstDash val="solid"/>
       <a:round/>
@@ -1485,7 +1485,7 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <plotArea>
       <layout/>
@@ -1495,7 +1495,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1503,12 +1503,12 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:schemeClr val="accent3">
                   <a:lumMod val="75000"/>
                 </a:schemeClr>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:ln w="19050">
                 <a:solidFill>
                   <a:schemeClr val="lt1"/>
                 </a:solidFill>
@@ -1520,13 +1520,13 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:schemeClr val="tx2">
                   <a:lumMod val="40000"/>
                   <a:lumOff val="60000"/>
                 </a:schemeClr>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:ln w="19050">
                 <a:solidFill>
                   <a:schemeClr val="lt1"/>
                 </a:solidFill>
@@ -1538,8 +1538,8 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:noFill/>
+              <a:ln w="19050">
                 <a:solidFill>
                   <a:schemeClr val="lt1"/>
                 </a:solidFill>
@@ -1583,8 +1583,8 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:noFill/>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:noFill/>
       <a:prstDash val="solid"/>
       <a:round/>
@@ -1594,7 +1594,7 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <plotArea>
       <layout/>
@@ -1604,7 +1604,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1612,12 +1612,12 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:schemeClr val="accent4">
                   <a:lumMod val="75000"/>
                 </a:schemeClr>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:ln w="19050">
                 <a:solidFill>
                   <a:schemeClr val="lt1"/>
                 </a:solidFill>
@@ -1629,13 +1629,13 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:schemeClr val="tx2">
                   <a:lumMod val="40000"/>
                   <a:lumOff val="60000"/>
                 </a:schemeClr>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:ln w="19050">
                 <a:solidFill>
                   <a:schemeClr val="lt1"/>
                 </a:solidFill>
@@ -1647,8 +1647,8 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:noFill/>
+              <a:ln w="19050">
                 <a:solidFill>
                   <a:schemeClr val="lt1"/>
                 </a:solidFill>
@@ -1692,8 +1692,8 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:noFill/>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:noFill/>
       <a:prstDash val="solid"/>
       <a:round/>
@@ -1703,7 +1703,7 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <plotArea>
       <layout/>
@@ -1713,7 +1713,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1721,10 +1721,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:schemeClr val="accent1"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:ln w="19050">
                 <a:solidFill>
                   <a:schemeClr val="lt1"/>
                 </a:solidFill>
@@ -1736,10 +1736,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:schemeClr val="tx1"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:ln w="19050">
                 <a:solidFill>
                   <a:schemeClr val="lt1"/>
                 </a:solidFill>
@@ -1751,8 +1751,8 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:noFill/>
+              <a:ln w="19050">
                 <a:solidFill>
                   <a:schemeClr val="lt1"/>
                 </a:solidFill>
@@ -1796,8 +1796,8 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:noFill/>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:noFill/>
       <a:prstDash val="solid"/>
       <a:round/>
@@ -1807,7 +1807,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>2</col>
@@ -1827,9 +1827,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1854,9 +1854,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1881,9 +1881,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1908,9 +1908,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1933,26 +1933,26 @@
       <nvPicPr>
         <cNvPr id="18" name="Immagine 17"/>
         <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:srcRect/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr bwMode="auto">
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:xfrm>
           <a:off x="7479031" y="92003"/>
           <a:ext cx="485425" cy="288997"/>
         </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+        <a:prstGeom prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:noFill/>
+        <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -1976,26 +1976,26 @@
       <nvPicPr>
         <cNvPr id="21" name="Immagine 20"/>
         <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:srcRect/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr bwMode="auto">
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:xfrm>
           <a:off x="7541420" y="12741117"/>
           <a:ext cx="433992" cy="271937"/>
         </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+        <a:prstGeom prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:noFill/>
+        <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -2019,26 +2019,26 @@
       <nvPicPr>
         <cNvPr id="3" name="Immagine 2"/>
         <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId7"/>
+        <a:srcRect/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr bwMode="auto">
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:xfrm>
           <a:off x="7570470" y="38593395"/>
           <a:ext cx="414942" cy="275747"/>
         </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+        <a:prstGeom prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:noFill/>
+        <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -4232,7 +4232,7 @@
         <v/>
       </c>
       <c r="D83" s="54">
-        <f>_xlfn.XLOOKUP(C83,$G$95:$G$104,$H$95:$H$104)*_xlfn.XLOOKUP(I92,$G$84:$G$87,$K$84:$K$87)</f>
+        <f>INDEX($H$95:$H$104,MATCH(C83,$G$95:$G$104,0))*INDEX($K$84:$K$87,MATCH(I92,$G$84:$G$87,0))</f>
         <v/>
       </c>
       <c r="E83" s="2" t="n"/>
@@ -4441,15 +4441,15 @@
       <c r="F89" s="2" t="n"/>
       <c r="G89" s="2" t="n"/>
       <c r="H89" s="28">
-        <f t="array" ref="H89">_xlfn.IFS(H88&lt;=H84,$G$84,AND(H88&lt;=H85,H88&gt;H84),$G$85,AND(H88&lt;=H86,H88&gt;H85),$G$86,H88&gt;H86,$G$87)</f>
+        <f>IF(H88&lt;=H84,$G$84,IF(AND(H88&lt;=H85,H88&gt;H84),$G$85,IF(AND(H88&lt;=H86,H88&gt;H85),$G$86,IF(H88&gt;H86,$G$87))))</f>
         <v/>
       </c>
       <c r="I89" s="28">
-        <f t="array" ref="I89">_xlfn.IFS(I88&lt;=I84,$G$84,AND(I88&lt;=I85,I88&gt;I84),$G$85,AND(I88&lt;=I86,I88&gt;I85),$G$86,I88&gt;I86,$G$87)</f>
+        <f>IF(I88&lt;=I84,$G$84,IF(AND(I88&lt;=I85,I88&gt;I84),$G$85,IF(AND(I88&lt;=I86,I88&gt;I85),$G$86,IF(I88&gt;I86,$G$87))))</f>
         <v/>
       </c>
       <c r="J89" s="28">
-        <f t="array" ref="J89">_xlfn.IFS(J88&lt;=J84,$G$84,AND(J88&lt;=J85,J88&gt;J84),$G$85,AND(J88&lt;=J86,J88&gt;J85),$G$86,J88&gt;J86,$G$87)</f>
+        <f>IF(J88&lt;=J84,$G$84,IF(AND(J88&lt;=J85,J88&gt;J84),$G$85,IF(AND(J88&lt;=J86,J88&gt;J85),$G$86,IF(J88&gt;J86,$G$87))))</f>
         <v/>
       </c>
       <c r="K89" s="2" t="n"/>
@@ -4469,15 +4469,15 @@
       <c r="F90" s="2" t="n"/>
       <c r="G90" s="2" t="n"/>
       <c r="H90" s="27">
-        <f>_xlfn.XLOOKUP(H89,$G$84:$G$87,$F$84:$F$87)</f>
+        <f>INDEX($F$84:$F$87,MATCH(H89,$G$84:$G$87,0))</f>
         <v/>
       </c>
       <c r="I90" s="27">
-        <f>_xlfn.XLOOKUP(I89,$G$84:$G$87,$F$84:$F$87)</f>
+        <f>INDEX($F$84:$F$87,MATCH(I89,$G$84:$G$87,0))</f>
         <v/>
       </c>
       <c r="J90" s="27">
-        <f>_xlfn.XLOOKUP(J89,$G$84:$G$87,$F$84:$F$87)</f>
+        <f>INDEX($F$84:$F$87,MATCH(J89,$G$84:$G$87,0))</f>
         <v/>
       </c>
       <c r="K90" s="2" t="n"/>
@@ -4520,7 +4520,7 @@
       <c r="G92" s="2" t="n"/>
       <c r="H92" s="2" t="n"/>
       <c r="I92" s="50">
-        <f>IFERROR(_xlfn.XLOOKUP(I91,$F$84:$F$87,G84:G87),_xlfn.XLOOKUP(MEDIAN(H90:J90),$F$84:$F$87,$G$84:$G$87))</f>
+        <f>IFERROR(INDEX(G84:G87,MATCH(I91,$F$84:$F$87,0)),INDEX($G$84:$G$87,MATCH(MEDIAN(H90:J90),$F$84:$F$87,0)))</f>
         <v/>
       </c>
       <c r="J92" s="2" t="n"/>
@@ -5770,7 +5770,7 @@
         <v/>
       </c>
       <c r="B14" s="87">
-        <f>_xlfn.XLOOKUP(Input!C135,Input!D119:H119,Input!D118:H118)</f>
+        <f>INDEX(Input.$D$118:$H$118,MATCH(Input!C135,Input.$D$119:$H$119,0))</f>
         <v/>
       </c>
       <c r="D14" s="14" t="n"/>

</xml_diff>

<commit_message>
fix: update financial statement analysis template setting decimal notation according to the italian standard
</commit_message>
<xml_diff>
--- a/plugins/fs-analysis/skills/analyzing-financial-statements/assets/template.xlsx
+++ b/plugins/fs-analysis/skills/analyzing-financial-statements/assets/template.xlsx
@@ -4483,7 +4483,7 @@
       <c r="B85" s="51" t="n"/>
       <c r="C85" s="2" t="n"/>
       <c r="D85" s="55">
-        <f>"0 € - "&amp;TEXT(D83,"[$-410]#,##0")&amp;" €"</f>
+        <f>"0 € - "&amp;SUBSTITUTE(TEXT(D83,"#,##0"),",",".")&amp;" €"</f>
         <v/>
       </c>
       <c r="E85" s="2" t="n"/>
@@ -6041,19 +6041,19 @@
     </row>
     <row r="24" ht="29.1" customHeight="1" s="183">
       <c r="A24" s="117">
-        <f>IFERROR(TEXT((Input!B8-Input!C8)/Input!C8,"[$-410]+0.00%;[$-410]-0.00%;[$-410]0.00%") &amp; " vs " &amp; TEXT(Input!C8,"[$-410]#,##0"),"n.d.")</f>
+        <f>IFERROR(SUBSTITUTE(TEXT((Input!B8-Input!C8)/Input!C8,"+0.00%;-0.00%;0.00%"),".",",")&amp;" vs "&amp;SUBSTITUTE(TEXT(Input!C8,"#,##0"),",","."),"n.d.")</f>
         <v/>
       </c>
       <c r="B24" s="117">
-        <f>IFERROR(TEXT((Input!B17-Input!C17)/Input!C17,"[$-410]+0.00%;[$-410]-0.00%;[$-410]0.00%") &amp; " vs " &amp; TEXT(Input!C17,"[$-410]#,##0"),"n.d.")</f>
+        <f>IFERROR(SUBSTITUTE(TEXT((Input!B17-Input!C17)/Input!C17,"+0.00%;-0.00%;0.00%"),".",",")&amp;" vs "&amp;SUBSTITUTE(TEXT(Input!C17,"#,##0"),",","."),"n.d.")</f>
         <v/>
       </c>
       <c r="C24" s="117">
-        <f>IFERROR(TEXT(((Input!B17+Input!B14)-(Input!C17+Input!C14))/(Input!C17+Input!C14),"[$-410]+0.00%;[$-410]-0.00%;[$-410]0.00%") &amp; " vs " &amp; TEXT((Input!C17+Input!C14),"[$-410]#,##0"),"n.d.")</f>
+        <f>IFERROR(SUBSTITUTE(TEXT(((Input!B17+Input!B14)-(Input!C17+Input!C14))/(Input!C17+Input!C14),"+0.00%;-0.00%;0.00%"),".",",")&amp;" vs "&amp;SUBSTITUTE(TEXT((Input!C17+Input!C14),"#,##0"),",","."),"n.d.")</f>
         <v/>
       </c>
       <c r="D24" s="117">
-        <f>IFERROR(TEXT((Input!B20-Input!C20)/Input!C20,"[$-410]+0.00%;[$-410]-0.00%;[$-410]0.00%") &amp; " vs " &amp; TEXT(Input!C20,"[$-410]#,##0"),"n.d.")</f>
+        <f>IFERROR(SUBSTITUTE(TEXT((Input!B20-Input!C20)/Input!C20,"+0.00%;-0.00%;0.00%"),".",",")&amp;" vs "&amp;SUBSTITUTE(TEXT(Input!C20,"#,##0"),",","."),"n.d.")</f>
         <v/>
       </c>
       <c r="E24" s="114" t="n"/>
@@ -6113,19 +6113,19 @@
     </row>
     <row r="28" ht="29.1" customHeight="1" s="183">
       <c r="A28" s="117">
-        <f>IFERROR(TEXT((Input!B34-Input!C34)/Input!C34,"[$-410]+0.00%;[$-410]-0.00%;[$-410]0.00%") &amp; " vs " &amp; TEXT(Input!C34,"[$-410]#,##0"),"n.d.")</f>
+        <f>IFERROR(SUBSTITUTE(TEXT((Input!B34-Input!C34)/Input!C34,"+0.00%;-0.00%;0.00%"),".",",")&amp;" vs "&amp;SUBSTITUTE(TEXT(Input!C34,"#,##0"),",","."),"n.d.")</f>
         <v/>
       </c>
       <c r="B28" s="117">
-        <f>IFERROR(TEXT((Input!B40-Input!C40)/Input!C40,"[$-410]+0.00%;[$-410]-0.00%;[$-410]0.00%")&amp;" vs "&amp;TEXT(Input!C40,"[$-410]#,##0"),"n.d.")</f>
+        <f>IFERROR(SUBSTITUTE(TEXT((Input!B40-Input!C40)/Input!C40,"+0.00%;-0.00%;0.00%"),".",",")&amp;" vs "&amp;SUBSTITUTE(TEXT(Input!C40,"#,##0"),",","."),"n.d.")</f>
         <v/>
       </c>
       <c r="C28" s="117">
-        <f>IFERROR(TEXT((Input!B31-Input!C31)/Input!C31,"[$-410]+0.00%;[$-410]-0.00%;[$-410]0.00%") &amp; " vs " &amp; TEXT(Input!C31,"[$-410]#,##0"),"n.d.")</f>
+        <f>IFERROR(SUBSTITUTE(TEXT((Input!B31-Input!C31)/Input!C31,"+0.00%;-0.00%;0.00%"),".",",")&amp;" vs "&amp;SUBSTITUTE(TEXT(Input!C31,"#,##0"),",","."),"n.d.")</f>
         <v/>
       </c>
       <c r="D28" s="117">
-        <f>IFERROR(TEXT((Input!B21-Input!C21)/Input!C21,"[$-410]+0.00%;[$-410]-0.00%;[$-410]0.00%") &amp; " vs " &amp; TEXT(Input!C21,"[$-410]#,##0"),"n.d.")</f>
+        <f>IFERROR(SUBSTITUTE(TEXT((Input!B21-Input!C21)/Input!C21,"+0.00%;-0.00%;0.00%"),".",",")&amp;" vs "&amp;SUBSTITUTE(TEXT(Input!C21,"#,##0"),",","."),"n.d.")</f>
         <v/>
       </c>
       <c r="E28" s="114" t="n"/>

</xml_diff>